<commit_message>
docs(measurements): add XY shrink and insert-length rows
Shrink cancels between printed parts but not where a print wraps a rigid
one: the pane rebate is pane + 2 x clearance, so 0.3 % along the 127 mm
pane uses up the whole 0.3 mm. A new Fit coupon row takes the coupon's
118 mm strip length; two computed rows turn it into a shrink percentage
and the pane clearance per side after shrink, flagged TIGHT under 0.1.
The summary count includes TIGHT.

Inserts gains the four insert lengths (insert38_len, insert_len, M4,
M3) with the model's hole depths in the notes. BRINGUP step 1 asks for
the strip measurement.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/measurements.xlsx
+++ b/docs/measurements.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K114"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1055,7 +1055,7 @@
         <f>IF(OR(H16="",I16=""),"",IF(ABS(H16)&gt;I16,IF(ISNUMBER(G16),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -1456,7 +1456,7 @@
         <f>IF(OR(H27="",I27=""),"",IF(ABS(H27)&gt;I27,IF(ISNUMBER(G27),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K27" s="5" t="inlineStr"/>
+      <c r="K27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -1526,7 +1526,7 @@
         <f>IF(OR(H29="",I29=""),"",IF(ABS(H29)&gt;I29,IF(ISNUMBER(G29),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K29" s="5" t="inlineStr"/>
+      <c r="K29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -1596,7 +1596,7 @@
         <f>IF(OR(H31="",I31=""),"",IF(ABS(H31)&gt;I31,IF(ISNUMBER(G31),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K31" s="5" t="inlineStr"/>
+      <c r="K31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
@@ -1736,7 +1736,7 @@
       <c r="D35" s="9" t="n">
         <v>1.778</v>
       </c>
-      <c r="E35" s="9" t="inlineStr"/>
+      <c r="E35" s="9" t="n"/>
       <c r="F35" s="8" t="n">
         <v>1.778</v>
       </c>
@@ -1822,7 +1822,7 @@
         <f>IF(OR(H37="",I37=""),"",IF(ABS(H37)&gt;I37,IF(ISNUMBER(G37),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K37" s="5" t="inlineStr"/>
+      <c r="K37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
@@ -1843,7 +1843,7 @@
       <c r="D38" s="9" t="n">
         <v>0.95</v>
       </c>
-      <c r="E38" s="9" t="inlineStr"/>
+      <c r="E38" s="9" t="n"/>
       <c r="F38" s="8" t="n">
         <v>0.95</v>
       </c>
@@ -1897,7 +1897,7 @@
         <f>IF(OR(H39="",I39=""),"",IF(ABS(H39)&gt;I39,IF(ISNUMBER(G39),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K39" s="5" t="inlineStr"/>
+      <c r="K39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
@@ -1953,7 +1953,7 @@
       <c r="D41" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="E41" s="9" t="inlineStr"/>
+      <c r="E41" s="9" t="n"/>
       <c r="F41" s="8" t="n"/>
       <c r="G41" s="11">
         <f>IF(AND(ISNUMBER(G39),ISNUMBER(G40),G39&gt;0),ROUND(2*G40/G39+1,2),"")</f>
@@ -2050,7 +2050,7 @@
         <f>IF(OR(H43="",I43=""),"",IF(ABS(H43)&gt;I43,IF(ISNUMBER(G43),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K43" s="5" t="inlineStr"/>
+      <c r="K43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
@@ -2409,7 +2409,7 @@
           <t>wart_l</t>
         </is>
       </c>
-      <c r="D53" s="9">
+      <c r="D53" s="9" t="n">
         <v>86</v>
       </c>
       <c r="E53" s="9" t="inlineStr">
@@ -2418,8 +2418,8 @@
         </is>
       </c>
       <c r="F53" s="8" t="n"/>
-      <c r="G53" s="10">
-        <v>85.6</v>
+      <c r="G53" s="10" t="n">
+        <v>85.59999999999999</v>
       </c>
       <c r="H53" s="9">
         <f>IF(NOT(ISNUMBER(D53)),"",IF(ISNUMBER(G53),G53-D53,IF(ISNUMBER(F53),F53-D53,"")))</f>
@@ -2454,7 +2454,7 @@
           <t>wart_w</t>
         </is>
       </c>
-      <c r="D54" s="9">
+      <c r="D54" s="9" t="n">
         <v>47</v>
       </c>
       <c r="E54" s="9" t="inlineStr">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="F54" s="8" t="n"/>
-      <c r="G54" s="10">
+      <c r="G54" s="10" t="n">
         <v>47</v>
       </c>
       <c r="H54" s="9">
@@ -2499,7 +2499,7 @@
           <t>wart_t</t>
         </is>
       </c>
-      <c r="D55" s="9">
+      <c r="D55" s="9" t="n">
         <v>35</v>
       </c>
       <c r="E55" s="9" t="inlineStr">
@@ -2549,7 +2549,7 @@
       <c r="F56" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="G56" s="10">
+      <c r="G56" s="10" t="n">
         <v>21</v>
       </c>
       <c r="H56" s="9">
@@ -2590,7 +2590,7 @@
       <c r="F57" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G57" s="10">
+      <c r="G57" s="10" t="n">
         <v>2.28</v>
       </c>
       <c r="H57" s="9">
@@ -2627,8 +2627,8 @@
         </is>
       </c>
       <c r="F58" s="8" t="n"/>
-      <c r="G58" s="10">
-        <v>1.0</v>
+      <c r="G58" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="H58" s="9">
         <f>IF(NOT(ISNUMBER(D58)),"",IF(ISNUMBER(G58),G58-D58,IF(ISNUMBER(F58),F58-D58,"")))</f>
@@ -2947,7 +2947,7 @@
         <f>IF(OR(H66="",I66=""),"",IF(ABS(H66)&gt;I66,IF(ISNUMBER(G66),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K66" s="5" t="inlineStr"/>
+      <c r="K66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
@@ -2986,7 +2986,7 @@
         <f>IF(OR(H67="",I67=""),"",IF(ABS(H67)&gt;I67,IF(ISNUMBER(G67),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K67" s="5" t="inlineStr"/>
+      <c r="K67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
@@ -3111,7 +3111,7 @@
         <f>IF(OR(H70="",I70=""),"",IF(ABS(H70)&gt;I70,IF(ISNUMBER(G70),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K70" s="5" t="inlineStr"/>
+      <c r="K70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="inlineStr">
@@ -3150,7 +3150,7 @@
         <f>IF(OR(H71="",I71=""),"",IF(ABS(H71)&gt;I71,IF(ISNUMBER(G71),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K71" s="5" t="inlineStr"/>
+      <c r="K71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="9" t="inlineStr">
@@ -3593,7 +3593,7 @@
         <f>IF(OR(H82="",I82=""),"",IF(ABS(H82)&gt;I82,IF(ISNUMBER(G82),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K82" s="5" t="inlineStr"/>
+      <c r="K82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="inlineStr">
@@ -3675,7 +3675,7 @@
         <f>IF(OR(H84="",I84=""),"",IF(ABS(H84)&gt;I84,IF(ISNUMBER(G84),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K84" s="5" t="inlineStr"/>
+      <c r="K84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="inlineStr">
@@ -3843,7 +3843,7 @@
         <f>IF(OR(H88="",I88=""),"",IF(ABS(H88)&gt;I88,IF(ISNUMBER(G88),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K88" s="5" t="inlineStr"/>
+      <c r="K88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="inlineStr">
@@ -3968,7 +3968,7 @@
         <f>IF(OR(H91="",I91=""),"",IF(ABS(H91)&gt;I91,IF(ISNUMBER(G91),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K91" s="5" t="inlineStr"/>
+      <c r="K91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
@@ -4007,7 +4007,7 @@
         <f>IF(OR(H92="",I92=""),"",IF(ABS(H92)&gt;I92,IF(ISNUMBER(G92),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K92" s="5" t="inlineStr"/>
+      <c r="K92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
@@ -4046,26 +4046,26 @@
         <f>IF(OR(H93="",I93=""),"",IF(ABS(H93)&gt;I93,IF(ISNUMBER(G93),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K93" s="5" t="inlineStr"/>
+      <c r="K93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="9" t="inlineStr">
         <is>
-          <t>Fit coupon</t>
+          <t>Inserts</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>General fit clearance</t>
+          <t>3/8-16 insert length</t>
         </is>
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>clearance</t>
+          <t>insert38_len</t>
         </is>
       </c>
       <c r="D94" s="9" t="n">
-        <v>0.3</v>
+        <v>12.7</v>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
         <v/>
       </c>
       <c r="I94" s="9" t="n">
-        <v>0.05</v>
+        <v>0.5</v>
       </c>
       <c r="J94" s="11">
         <f>IF(OR(H94="",I94=""),"",IF(ABS(H94)&gt;I94,IF(ISNUMBER(G94),"UPDATE","UPDATE (spec)"),"ok"))</f>
@@ -4087,23 +4087,29 @@
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
-          <t>Adjust after the coupon: keyhole, pane slot, screw pilots.</t>
+          <t>From the insert datasheet. The tripod pad hole is this deep plus 1 and the pad sits flush with the floor ribs, so a longer insert needs a deeper pad.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="9" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Inserts</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Distance from the case position to the projection surface</t>
-        </is>
-      </c>
-      <c r="C95" s="9" t="n"/>
-      <c r="D95" s="9" t="n"/>
+          <t>1/4-20 insert length</t>
+        </is>
+      </c>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>insert_len</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="n">
+        <v>9</v>
+      </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
           <t>mm</t>
@@ -4115,26 +4121,28 @@
         <f>IF(NOT(ISNUMBER(D95)),"",IF(ISNUMBER(G95),G95-D95,IF(ISNUMBER(F95),F95-D95,"")))</f>
         <v/>
       </c>
-      <c r="I95" s="9" t="n"/>
+      <c r="I95" s="9" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J95" s="11">
         <f>IF(OR(H95="",I95=""),"",IF(ABS(H95)&gt;I95,IF(ISNUMBER(G95),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
-          <t>Lens face to the surface, straight on, case where it will stand.</t>
+          <t>Pedestal column hole and the 1/4-20 tripod hole are this deep. A longer insert bottoms out before it seats.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="9" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Inserts</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>Projection surface: bottom edge height above ground</t>
+          <t>M4 insert length</t>
         </is>
       </c>
       <c r="C96" s="9" t="n"/>
@@ -4155,17 +4163,21 @@
         <f>IF(OR(H96="",I96=""),"",IF(ABS(H96)&gt;I96,IF(ISNUMBER(G96),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K96" s="5" t="inlineStr"/>
+      <c r="K96" s="5" t="inlineStr">
+        <is>
+          <t>Hatch stud holes are 8 deep into the wall bosses; an insert over about 7.5 breaks through.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="9" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Inserts</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>Projection surface: top edge height above ground</t>
+          <t>M3 insert length</t>
         </is>
       </c>
       <c r="C97" s="9" t="n"/>
@@ -4186,21 +4198,31 @@
         <f>IF(OR(H97="",I97=""),"",IF(ABS(H97)&gt;I97,IF(ISNUMBER(G97),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K97" s="5" t="inlineStr"/>
+      <c r="K97" s="5" t="inlineStr">
+        <is>
+          <t>Sled thumbscrew hole in the floor is 6 deep.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="9" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Fit coupon</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>Projection surface width</t>
-        </is>
-      </c>
-      <c r="C98" s="9" t="n"/>
-      <c r="D98" s="9" t="n"/>
+          <t>General fit clearance</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>clearance</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="n">
+        <v>0.3</v>
+      </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
           <t>mm</t>
@@ -4212,35 +4234,33 @@
         <f>IF(NOT(ISNUMBER(D98)),"",IF(ISNUMBER(G98),G98-D98,IF(ISNUMBER(F98),F98-D98,"")))</f>
         <v/>
       </c>
-      <c r="I98" s="9" t="n"/>
+      <c r="I98" s="9" t="n">
+        <v>0.05</v>
+      </c>
       <c r="J98" s="11">
         <f>IF(OR(H98="",I98=""),"",IF(ABS(H98)&gt;I98,IF(ISNUMBER(G98),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
       <c r="K98" s="5" t="inlineStr">
         <is>
-          <t>Compare with the computed image width below.</t>
+          <t>Adjust after the coupon: keyhole, pane slot, screw pilots.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="9" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Fit coupon</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>Lens height above ground, case on its feet</t>
-        </is>
-      </c>
-      <c r="C99" s="9" t="inlineStr">
-        <is>
-          <t>(z_lens)</t>
-        </is>
-      </c>
+          <t>XY shrink: coupon strip length</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="n"/>
       <c r="D99" s="9" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
@@ -4254,7 +4274,7 @@
         <v/>
       </c>
       <c r="I99" s="9" t="n">
-        <v>5</v>
+        <v>0.35</v>
       </c>
       <c r="J99" s="11">
         <f>IF(OR(H99="",I99=""),"",IF(ABS(H99)&gt;I99,IF(ISNUMBER(G99),"UPDATE","UPDATE (spec)"),"ok"))</f>
@@ -4262,31 +4282,31 @@
       </c>
       <c r="K99" s="5" t="inlineStr">
         <is>
-          <t>From the model: feet 6 + floor 6 + pedestal 30 + ball head 40 + lens_z 33. Measure it once assembled.</t>
+          <t>Measure the 118 mm strip once it is cool. Shrink cancels between printed parts (lid on base, tile seams) but not where a print wraps a rigid part: the pane rebate is pane + 2 x clearance, so 0.3 % along the 127 mm pane eats the whole 0.3 clearance. The two rows below work it out.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Fit coupon</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>Image width at that distance</t>
+          <t>XY shrink</t>
         </is>
       </c>
       <c r="C100" s="9" t="n"/>
       <c r="D100" s="9" t="n"/>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F100" s="8" t="n"/>
       <c r="G100" s="11">
-        <f>IF(ISNUMBER(G95),ROUND(G95/IF(ISNUMBER(G38),G38,D38),0),"")</f>
+        <f>IF(AND(ISNUMBER(G99),G99&gt;0),ROUND((D99-G99)/D99*100,2),"")</f>
         <v/>
       </c>
       <c r="H100" s="9">
@@ -4300,19 +4320,19 @@
       </c>
       <c r="K100" s="5" t="inlineStr">
         <is>
-          <t>Computed: distance / throw ratio (measured if filled, else default). Do not type here.</t>
+          <t>Computed from the strip. Do not type here.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="9" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Fit coupon</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>Image centre height above ground</t>
+          <t>Pane clearance after shrink, per side</t>
         </is>
       </c>
       <c r="C101" s="9" t="n"/>
@@ -4324,21 +4344,21 @@
       </c>
       <c r="F101" s="8" t="n"/>
       <c r="G101" s="11">
-        <f>IF(AND(ISNUMBER(G96),ISNUMBER(G97)),(G96+G97)/2,"")</f>
+        <f>IF(ISNUMBER(G100),ROUND(((IF(ISNUMBER(G87),G87,D87)+2*IF(ISNUMBER(G98),G98,D98))*(1-G100/100)-IF(ISNUMBER(G87),G87,D87))/2,2),"")</f>
         <v/>
       </c>
       <c r="H101" s="9">
-        <f>IF(NOT(ISNUMBER(D101)),"",IF(ISNUMBER(G101),G101-D101,IF(ISNUMBER(F101),F101-D101,"")))</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="I101" s="9" t="n"/>
       <c r="J101" s="11">
-        <f>IF(OR(H101="",I101=""),"",IF(ABS(H101)&gt;I101,IF(ISNUMBER(G101),"UPDATE","UPDATE (spec)"),"ok"))</f>
+        <f>IF(NOT(ISNUMBER(G101)),"",IF(G101&lt;0.1,"TIGHT","ok"))</f>
         <v/>
       </c>
       <c r="K101" s="5" t="inlineStr">
         <is>
-          <t>Computed from the two edge heights. Do not type here.</t>
+          <t>Computed: (pane + 2 x clearance) x (1 - shrink) - pane, halved. TIGHT under 0.1: scale the window frame and base front by 118 / strip in the slicer, or add the shortfall to pane_w and pane_h. Do not type here.</t>
         </is>
       </c>
     </row>
@@ -4350,39 +4370,30 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>Tilt needed to centre the image</t>
-        </is>
-      </c>
-      <c r="C102" s="9" t="inlineStr">
-        <is>
-          <t>cone_tilt</t>
-        </is>
-      </c>
-      <c r="D102" s="9" t="n">
-        <v>12</v>
-      </c>
+          <t>Distance from the case position to the projection surface</t>
+        </is>
+      </c>
+      <c r="C102" s="9" t="n"/>
+      <c r="D102" s="9" t="n"/>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>deg</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="F102" s="8" t="n"/>
-      <c r="G102" s="11">
-        <f>IF(AND(ISNUMBER(G95),ISNUMBER(G101),G95&gt;0),ROUND(DEGREES(ATAN((G101-IF(ISNUMBER(G99),G99,D99))/G95)),1),"")</f>
-        <v/>
-      </c>
+      <c r="G102" s="10" t="n"/>
       <c r="H102" s="9">
-        <f>IF(ISNUMBER(G102),G102-D102,"")</f>
+        <f>IF(NOT(ISNUMBER(D102)),"",IF(ISNUMBER(G102),G102-D102,IF(ISNUMBER(F102),F102-D102,"")))</f>
         <v/>
       </c>
       <c r="I102" s="9" t="n"/>
       <c r="J102" s="11">
-        <f>IF(NOT(ISNUMBER(G102)),"",IF(OR(G102&gt;D102,G102&lt;-15),"OVER LIMIT","ok"))</f>
+        <f>IF(OR(H102="",I102=""),"",IF(ABS(H102)&gt;I102,IF(ISNUMBER(G102),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
       <c r="K102" s="5" t="inlineStr">
         <is>
-          <t>Computed. Limit is cone_tilt (12) up and aim_max (15) down before the light cone clips the visor or the body hits the head. OVER LIMIT means a riser, the tripod or a longer throw. Do not type here.</t>
+          <t>Lens face to the surface, straight on, case where it will stand.</t>
         </is>
       </c>
     </row>
@@ -4394,14 +4405,14 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Ground slope at the case position</t>
+          <t>Projection surface: bottom edge height above ground</t>
         </is>
       </c>
       <c r="C103" s="9" t="n"/>
       <c r="D103" s="9" t="n"/>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>deg</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="F103" s="8" t="n"/>
@@ -4415,11 +4426,7 @@
         <f>IF(OR(H103="",I103=""),"",IF(ABS(H103)&gt;I103,IF(ISNUMBER(G103),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K103" s="5" t="inlineStr">
-        <is>
-          <t>Adds to the tilt. Shim the feet or use the tripod.</t>
-        </is>
-      </c>
+      <c r="K103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="9" t="inlineStr">
@@ -4429,14 +4436,14 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>Distance from the case to where visitors first appear</t>
+          <t>Projection surface: top edge height above ground</t>
         </is>
       </c>
       <c r="C104" s="9" t="n"/>
       <c r="D104" s="9" t="n"/>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="F104" s="8" t="n"/>
@@ -4450,11 +4457,7 @@
         <f>IF(OR(H104="",I104=""),"",IF(ABS(H104)&gt;I104,IF(ISNUMBER(G104),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K104" s="5" t="inlineStr">
-        <is>
-          <t>HC-SR501 range is about 7 m. Sets the PIR sensitivity and whether the rear wall is the right face for it.</t>
-        </is>
-      </c>
+      <c r="K104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="9" t="inlineStr">
@@ -4464,14 +4467,14 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>Distance from the case to the GFCI outlet</t>
+          <t>Projection surface width</t>
         </is>
       </c>
       <c r="C105" s="9" t="n"/>
       <c r="D105" s="9" t="n"/>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="F105" s="8" t="n"/>
@@ -4487,28 +4490,28 @@
       </c>
       <c r="K105" s="5" t="inlineStr">
         <is>
-          <t>One AC cord, under a cord cover across any path. Sets its length.</t>
+          <t>Compare with the computed image width below.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="9" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>Centre of mass behind the footprint centre (+ = rear)</t>
+          <t>Lens height above ground, case on its feet</t>
         </is>
       </c>
       <c r="C106" s="9" t="inlineStr">
         <is>
-          <t>tripod_y</t>
+          <t>(z_lens)</t>
         </is>
       </c>
       <c r="D106" s="9" t="n">
-        <v>5</v>
+        <v>115</v>
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
@@ -4530,82 +4533,350 @@
       </c>
       <c r="K106" s="5" t="inlineStr">
         <is>
+          <t>From the model: feet 6 + floor 6 + pedestal 30 + ball head 40 + lens_z 33. Measure it once assembled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="9" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Image width at that distance</t>
+        </is>
+      </c>
+      <c r="C107" s="9" t="n"/>
+      <c r="D107" s="9" t="n"/>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F107" s="8" t="n"/>
+      <c r="G107" s="11">
+        <f>IF(ISNUMBER(G102),ROUND(G102/IF(ISNUMBER(G38),G38,D38),0),"")</f>
+        <v/>
+      </c>
+      <c r="H107" s="9">
+        <f>IF(NOT(ISNUMBER(D107)),"",IF(ISNUMBER(G107),G107-D107,IF(ISNUMBER(F107),F107-D107,"")))</f>
+        <v/>
+      </c>
+      <c r="I107" s="9" t="n"/>
+      <c r="J107" s="11">
+        <f>IF(OR(H107="",I107=""),"",IF(ABS(H107)&gt;I107,IF(ISNUMBER(G107),"UPDATE","UPDATE (spec)"),"ok"))</f>
+        <v/>
+      </c>
+      <c r="K107" s="5" t="inlineStr">
+        <is>
+          <t>Computed: distance / throw ratio (measured if filled, else default). Do not type here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="9" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Image centre height above ground</t>
+        </is>
+      </c>
+      <c r="C108" s="9" t="n"/>
+      <c r="D108" s="9" t="n"/>
+      <c r="E108" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F108" s="8" t="n"/>
+      <c r="G108" s="11">
+        <f>IF(AND(ISNUMBER(G103),ISNUMBER(G104)),(G103+G104)/2,"")</f>
+        <v/>
+      </c>
+      <c r="H108" s="9">
+        <f>IF(NOT(ISNUMBER(D108)),"",IF(ISNUMBER(G108),G108-D108,IF(ISNUMBER(F108),F108-D108,"")))</f>
+        <v/>
+      </c>
+      <c r="I108" s="9" t="n"/>
+      <c r="J108" s="11">
+        <f>IF(OR(H108="",I108=""),"",IF(ABS(H108)&gt;I108,IF(ISNUMBER(G108),"UPDATE","UPDATE (spec)"),"ok"))</f>
+        <v/>
+      </c>
+      <c r="K108" s="5" t="inlineStr">
+        <is>
+          <t>Computed from the two edge heights. Do not type here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="9" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Tilt needed to centre the image</t>
+        </is>
+      </c>
+      <c r="C109" s="9" t="inlineStr">
+        <is>
+          <t>cone_tilt</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+      <c r="F109" s="8" t="n"/>
+      <c r="G109" s="11">
+        <f>IF(AND(ISNUMBER(G102),ISNUMBER(G108),G102&gt;0),ROUND(DEGREES(ATAN((G108-IF(ISNUMBER(G106),G106,D106))/G102)),1),"")</f>
+        <v/>
+      </c>
+      <c r="H109" s="9">
+        <f>IF(ISNUMBER(G109),G109-D109,"")</f>
+        <v/>
+      </c>
+      <c r="I109" s="9" t="n"/>
+      <c r="J109" s="11">
+        <f>IF(NOT(ISNUMBER(G109)),"",IF(OR(G109&gt;D109,G109&lt;-15),"OVER LIMIT","ok"))</f>
+        <v/>
+      </c>
+      <c r="K109" s="5" t="inlineStr">
+        <is>
+          <t>Computed. Limit is cone_tilt (12) up and aim_max (15) down before the light cone clips the visor or the body hits the head. OVER LIMIT means a riser, the tripod or a longer throw. Do not type here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="9" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>Ground slope at the case position</t>
+        </is>
+      </c>
+      <c r="C110" s="9" t="n"/>
+      <c r="D110" s="9" t="n"/>
+      <c r="E110" s="9" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+      <c r="F110" s="8" t="n"/>
+      <c r="G110" s="10" t="n"/>
+      <c r="H110" s="9">
+        <f>IF(NOT(ISNUMBER(D110)),"",IF(ISNUMBER(G110),G110-D110,IF(ISNUMBER(F110),F110-D110,"")))</f>
+        <v/>
+      </c>
+      <c r="I110" s="9" t="n"/>
+      <c r="J110" s="11">
+        <f>IF(OR(H110="",I110=""),"",IF(ABS(H110)&gt;I110,IF(ISNUMBER(G110),"UPDATE","UPDATE (spec)"),"ok"))</f>
+        <v/>
+      </c>
+      <c r="K110" s="5" t="inlineStr">
+        <is>
+          <t>Adds to the tilt. Shim the feet or use the tripod.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="9" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Distance from the case to where visitors first appear</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="n"/>
+      <c r="D111" s="9" t="n"/>
+      <c r="E111" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F111" s="8" t="n"/>
+      <c r="G111" s="10" t="n"/>
+      <c r="H111" s="9">
+        <f>IF(NOT(ISNUMBER(D111)),"",IF(ISNUMBER(G111),G111-D111,IF(ISNUMBER(F111),F111-D111,"")))</f>
+        <v/>
+      </c>
+      <c r="I111" s="9" t="n"/>
+      <c r="J111" s="11">
+        <f>IF(OR(H111="",I111=""),"",IF(ABS(H111)&gt;I111,IF(ISNUMBER(G111),"UPDATE","UPDATE (spec)"),"ok"))</f>
+        <v/>
+      </c>
+      <c r="K111" s="5" t="inlineStr">
+        <is>
+          <t>HC-SR501 range is about 7 m. Sets the PIR sensitivity and whether the rear wall is the right face for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="9" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>Distance from the case to the GFCI outlet</t>
+        </is>
+      </c>
+      <c r="C112" s="9" t="n"/>
+      <c r="D112" s="9" t="n"/>
+      <c r="E112" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F112" s="8" t="n"/>
+      <c r="G112" s="10" t="n"/>
+      <c r="H112" s="9">
+        <f>IF(NOT(ISNUMBER(D112)),"",IF(ISNUMBER(G112),G112-D112,IF(ISNUMBER(F112),F112-D112,"")))</f>
+        <v/>
+      </c>
+      <c r="I112" s="9" t="n"/>
+      <c r="J112" s="11">
+        <f>IF(OR(H112="",I112=""),"",IF(ABS(H112)&gt;I112,IF(ISNUMBER(G112),"UPDATE","UPDATE (spec)"),"ok"))</f>
+        <v/>
+      </c>
+      <c r="K112" s="5" t="inlineStr">
+        <is>
+          <t>One AC cord, under a cord cover across any path. Sets its length.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="9" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Centre of mass behind the footprint centre (+ = rear)</t>
+        </is>
+      </c>
+      <c r="C113" s="9" t="inlineStr">
+        <is>
+          <t>tripod_y</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E113" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F113" s="8" t="n"/>
+      <c r="G113" s="10" t="n"/>
+      <c r="H113" s="9">
+        <f>IF(NOT(ISNUMBER(D113)),"",IF(ISNUMBER(G113),G113-D113,IF(ISNUMBER(F113),F113-D113,"")))</f>
+        <v/>
+      </c>
+      <c r="I113" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J113" s="11">
+        <f>IF(OR(H113="",I113=""),"",IF(ABS(H113)&gt;I113,IF(ISNUMBER(G113),"UPDATE","UPDATE (spec)"),"ok"))</f>
+        <v/>
+      </c>
+      <c r="K113" s="5" t="inlineStr">
+        <is>
           <t>Loaded case, lid on: balance it on a rod across the feet, mark the line, measure from the footprint centre. Move tripod_y and reprint the base rear tile only if it moves more than the tolerance.</t>
         </is>
       </c>
     </row>
-    <row r="107"/>
-    <row r="108">
-      <c r="A108" s="6" t="inlineStr">
+    <row r="114"/>
+    <row r="115">
+      <c r="A115" s="6" t="inlineStr">
         <is>
           <t>Parameters to update</t>
         </is>
       </c>
-      <c r="B108" s="6">
-        <f>COUNTIF(J7:J106,"UPDATE*")+COUNTIF(J7:J106,"OVER LIMIT")</f>
-        <v/>
-      </c>
-      <c r="C108" s="6" t="inlineStr">
+      <c r="B115" s="6">
+        <f>COUNTIF(J7:J113,"UPDATE*")+COUNTIF(J7:J113,"OVER LIMIT")+COUNTIF(J7:J113,"TIGHT")</f>
+        <v/>
+      </c>
+      <c r="C115" s="6" t="inlineStr">
         <is>
           <t>Rows still blank</t>
         </is>
       </c>
-      <c r="D108" s="6">
-        <f>COUNTBLANK(G7:G106)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="109"/>
-    <row r="110">
-      <c r="A110" s="6" t="inlineStr">
+      <c r="D115" s="6">
+        <f>COUNTBLANK(G7:G113)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116"/>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
         <is>
           <t>Yellow cell</t>
         </is>
       </c>
-      <c r="B111" s="4" t="inlineStr">
+      <c r="B118" s="4" t="inlineStr">
         <is>
           <t>Type your measurement here.</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="8" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="8" t="inlineStr">
         <is>
           <t>Green value</t>
         </is>
       </c>
-      <c r="B112" s="4" t="inlineStr">
+      <c r="B119" s="4" t="inlineStr">
         <is>
           <t>From the Tkisko TO2 manual (manuals.plus, Oct 2022), its label and product photos. Confirm with calipers.</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="6" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="6" t="inlineStr">
         <is>
           <t>Bold value</t>
         </is>
       </c>
-      <c r="B113" s="4" t="inlineStr">
+      <c r="B120" s="4" t="inlineStr">
         <is>
           <t>Computed by the sheet. Leave it alone.</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
+    <row r="121">
+      <c r="A121" t="inlineStr">
         <is>
           <t>Defaults and tolerances</t>
         </is>
       </c>
-      <c r="B114" s="4" t="inlineStr">
+      <c r="B121" s="4" t="inlineStr">
         <is>
           <t>Taken from projector_pi_case.scad (v0.9 draft) and docs/BRINGUP.md. The weight default (720 g) is an assumption from the design log, not a measurement. Site rows and the Assembly row are about where the case will stand, not the hardware: fill them before printing the big tiles.</t>
         </is>

</xml_diff>

<commit_message>
feat(base): drop the tripod mount; the case sits flush on the ground
Remove the 3/8-16 and 1/4-20 inserts, their boss and the pad under the
floor. The case is ground-standing for this use and the projector has
its own ball head for aiming, so coarse aim is turning or shimming the
case. The fit coupon loses the 3/8 hole and shrinks one pitch.

Docs follow: BOM (no 3/8 insert, one 1/4-20), AIMING, ASSEMBLY,
BRINGUP, PRINTING (re-sliced coupon and base_front), README, CLAUDE.md,
DESIGN_LOG, and the measurements worksheet (insert38_d, tripod_y and
the 3/8 fit rows removed, formulas re-pointed).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/measurements.xlsx
+++ b/docs/measurements.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K114"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>(tripod_y centroid)</t>
+          <t/>
         </is>
       </c>
       <c r="D34" s="9" t="n">
@@ -3896,16 +3896,16 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>3/8-16 heat-set insert hole</t>
+          <t>1/4-20 heat-set insert hole</t>
         </is>
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>insert38_d</t>
+          <t>insert_d</t>
         </is>
       </c>
       <c r="D90" s="9" t="n">
-        <v>12.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
@@ -3925,11 +3925,7 @@
         <f>IF(OR(H90="",I90=""),"",IF(ABS(H90)&gt;I90,IF(ISNUMBER(G90),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K90" s="5" t="inlineStr">
-        <is>
-          <t>From the insert datasheet, then confirm on the fit coupon.</t>
-        </is>
-      </c>
+      <c r="K90" s="5" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
@@ -3939,16 +3935,16 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>1/4-20 heat-set insert hole</t>
+          <t>M4 heat-set insert hole</t>
         </is>
       </c>
       <c r="C91" s="9" t="inlineStr">
         <is>
-          <t>insert_d</t>
+          <t>m4_insert_d</t>
         </is>
       </c>
       <c r="D91" s="9" t="n">
-        <v>8.199999999999999</v>
+        <v>5.6</v>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
@@ -3978,16 +3974,16 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>M4 heat-set insert hole</t>
+          <t>M3 heat-set insert hole</t>
         </is>
       </c>
       <c r="C92" s="9" t="inlineStr">
         <is>
-          <t>m4_insert_d</t>
+          <t>m3_insert_d</t>
         </is>
       </c>
       <c r="D92" s="9" t="n">
-        <v>5.6</v>
+        <v>4</v>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
@@ -4012,21 +4008,21 @@
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>Inserts</t>
+          <t>Fit coupon</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>M3 heat-set insert hole</t>
+          <t>General fit clearance</t>
         </is>
       </c>
       <c r="C93" s="9" t="inlineStr">
         <is>
-          <t>m3_insert_d</t>
+          <t>clearance</t>
         </is>
       </c>
       <c r="D93" s="9" t="n">
-        <v>4</v>
+        <v>0.3</v>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
@@ -4040,33 +4036,31 @@
         <v/>
       </c>
       <c r="I93" s="9" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="J93" s="11">
         <f>IF(OR(H93="",I93=""),"",IF(ABS(H93)&gt;I93,IF(ISNUMBER(G93),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K93" s="5" t="inlineStr"/>
+      <c r="K93" s="5" t="inlineStr">
+        <is>
+          <t>Adjust after the coupon: keyhole, pane slot, screw pilots.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="9" t="inlineStr">
         <is>
-          <t>Fit coupon</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>General fit clearance</t>
-        </is>
-      </c>
-      <c r="C94" s="9" t="inlineStr">
-        <is>
-          <t>clearance</t>
-        </is>
-      </c>
-      <c r="D94" s="9" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Distance from the case position to the projection surface</t>
+        </is>
+      </c>
+      <c r="C94" s="9" t="n"/>
+      <c r="D94" s="9" t="n"/>
       <c r="E94" s="9" t="inlineStr">
         <is>
           <t>mm</t>
@@ -4078,16 +4072,14 @@
         <f>IF(NOT(ISNUMBER(D94)),"",IF(ISNUMBER(G94),G94-D94,IF(ISNUMBER(F94),F94-D94,"")))</f>
         <v/>
       </c>
-      <c r="I94" s="9" t="n">
-        <v>0.05</v>
-      </c>
+      <c r="I94" s="9" t="n"/>
       <c r="J94" s="11">
         <f>IF(OR(H94="",I94=""),"",IF(ABS(H94)&gt;I94,IF(ISNUMBER(G94),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
-          <t>Adjust after the coupon: keyhole, pane slot, screw pilots.</t>
+          <t>Lens face to the surface, straight on, case where it will stand.</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4091,7 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Distance from the case position to the projection surface</t>
+          <t>Projection surface: bottom edge height above ground</t>
         </is>
       </c>
       <c r="C95" s="9" t="n"/>
@@ -4120,11 +4112,7 @@
         <f>IF(OR(H95="",I95=""),"",IF(ABS(H95)&gt;I95,IF(ISNUMBER(G95),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K95" s="5" t="inlineStr">
-        <is>
-          <t>Lens face to the surface, straight on, case where it will stand.</t>
-        </is>
-      </c>
+      <c r="K95" s="5" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="9" t="inlineStr">
@@ -4134,7 +4122,7 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>Projection surface: bottom edge height above ground</t>
+          <t>Projection surface: top edge height above ground</t>
         </is>
       </c>
       <c r="C96" s="9" t="n"/>
@@ -4165,7 +4153,7 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>Projection surface: top edge height above ground</t>
+          <t>Projection surface width</t>
         </is>
       </c>
       <c r="C97" s="9" t="n"/>
@@ -4186,7 +4174,11 @@
         <f>IF(OR(H97="",I97=""),"",IF(ABS(H97)&gt;I97,IF(ISNUMBER(G97),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K97" s="5" t="inlineStr"/>
+      <c r="K97" s="5" t="inlineStr">
+        <is>
+          <t>Compare with the computed image width below.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="9" t="inlineStr">
@@ -4196,11 +4188,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>Projection surface width</t>
-        </is>
-      </c>
-      <c r="C98" s="9" t="n"/>
-      <c r="D98" s="9" t="n"/>
+          <t>Lens height above ground, case on its feet</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>(z_lens)</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="n">
+        <v>115</v>
+      </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
           <t>mm</t>
@@ -4212,14 +4210,16 @@
         <f>IF(NOT(ISNUMBER(D98)),"",IF(ISNUMBER(G98),G98-D98,IF(ISNUMBER(F98),F98-D98,"")))</f>
         <v/>
       </c>
-      <c r="I98" s="9" t="n"/>
+      <c r="I98" s="9" t="n">
+        <v>5</v>
+      </c>
       <c r="J98" s="11">
         <f>IF(OR(H98="",I98=""),"",IF(ABS(H98)&gt;I98,IF(ISNUMBER(G98),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
       <c r="K98" s="5" t="inlineStr">
         <is>
-          <t>Compare with the computed image width below.</t>
+          <t>From the model: feet 6 + floor 6 + pedestal 30 + ball head 40 + lens_z 33. Measure it once assembled.</t>
         </is>
       </c>
     </row>
@@ -4231,38 +4231,33 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>Lens height above ground, case on its feet</t>
-        </is>
-      </c>
-      <c r="C99" s="9" t="inlineStr">
-        <is>
-          <t>(z_lens)</t>
-        </is>
-      </c>
-      <c r="D99" s="9" t="n">
-        <v>115</v>
-      </c>
+          <t>Image width at that distance</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="n"/>
+      <c r="D99" s="9" t="n"/>
       <c r="E99" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
       <c r="F99" s="8" t="n"/>
-      <c r="G99" s="10" t="n"/>
+      <c r="G99" s="11">
+        <f>IF(ISNUMBER(G94),ROUND(G94/IF(ISNUMBER(G38),G38,D38),0),"")</f>
+        <v/>
+      </c>
       <c r="H99" s="9">
         <f>IF(NOT(ISNUMBER(D99)),"",IF(ISNUMBER(G99),G99-D99,IF(ISNUMBER(F99),F99-D99,"")))</f>
         <v/>
       </c>
-      <c r="I99" s="9" t="n">
-        <v>5</v>
-      </c>
+      <c r="I99" s="9" t="n"/>
       <c r="J99" s="11">
         <f>IF(OR(H99="",I99=""),"",IF(ABS(H99)&gt;I99,IF(ISNUMBER(G99),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
       <c r="K99" s="5" t="inlineStr">
         <is>
-          <t>From the model: feet 6 + floor 6 + pedestal 30 + ball head 40 + lens_z 33. Measure it once assembled.</t>
+          <t>Computed: distance / throw ratio (measured if filled, else default). Do not type here.</t>
         </is>
       </c>
     </row>
@@ -4274,7 +4269,7 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>Image width at that distance</t>
+          <t>Image centre height above ground</t>
         </is>
       </c>
       <c r="C100" s="9" t="n"/>
@@ -4286,7 +4281,7 @@
       </c>
       <c r="F100" s="8" t="n"/>
       <c r="G100" s="11">
-        <f>IF(ISNUMBER(G95),ROUND(G95/IF(ISNUMBER(G38),G38,D38),0),"")</f>
+        <f>IF(AND(ISNUMBER(G95),ISNUMBER(G96)),(G95+G96)/2,"")</f>
         <v/>
       </c>
       <c r="H100" s="9">
@@ -4300,7 +4295,7 @@
       </c>
       <c r="K100" s="5" t="inlineStr">
         <is>
-          <t>Computed: distance / throw ratio (measured if filled, else default). Do not type here.</t>
+          <t>Computed from the two edge heights. Do not type here.</t>
         </is>
       </c>
     </row>
@@ -4312,33 +4307,39 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>Image centre height above ground</t>
-        </is>
-      </c>
-      <c r="C101" s="9" t="n"/>
-      <c r="D101" s="9" t="n"/>
+          <t>Tilt needed to centre the image</t>
+        </is>
+      </c>
+      <c r="C101" s="9" t="inlineStr">
+        <is>
+          <t>cone_tilt</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="n">
+        <v>12</v>
+      </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>deg</t>
         </is>
       </c>
       <c r="F101" s="8" t="n"/>
       <c r="G101" s="11">
-        <f>IF(AND(ISNUMBER(G96),ISNUMBER(G97)),(G96+G97)/2,"")</f>
+        <f>IF(AND(ISNUMBER(G94),ISNUMBER(G100),G94&gt;0),ROUND(DEGREES(ATAN((G100-IF(ISNUMBER(G98),G98,D98))/G94)),1),"")</f>
         <v/>
       </c>
       <c r="H101" s="9">
-        <f>IF(NOT(ISNUMBER(D101)),"",IF(ISNUMBER(G101),G101-D101,IF(ISNUMBER(F101),F101-D101,"")))</f>
+        <f>IF(ISNUMBER(G101),G101-D101,"")</f>
         <v/>
       </c>
       <c r="I101" s="9" t="n"/>
       <c r="J101" s="11">
-        <f>IF(OR(H101="",I101=""),"",IF(ABS(H101)&gt;I101,IF(ISNUMBER(G101),"UPDATE","UPDATE (spec)"),"ok"))</f>
+        <f>IF(NOT(ISNUMBER(G101)),"",IF(OR(G101&gt;D101,G101&lt;-15),"OVER LIMIT","ok"))</f>
         <v/>
       </c>
       <c r="K101" s="5" t="inlineStr">
         <is>
-          <t>Computed from the two edge heights. Do not type here.</t>
+          <t>Computed. Limit is cone_tilt (12) up and aim_max (15) down before the light cone clips the visor or the body hits the head. OVER LIMIT means a riser or a longer throw. Do not type here.</t>
         </is>
       </c>
     </row>
@@ -4350,39 +4351,30 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>Tilt needed to centre the image</t>
-        </is>
-      </c>
-      <c r="C102" s="9" t="inlineStr">
-        <is>
-          <t>cone_tilt</t>
-        </is>
-      </c>
-      <c r="D102" s="9" t="n">
-        <v>12</v>
-      </c>
+          <t>Ground slope at the case position</t>
+        </is>
+      </c>
+      <c r="C102" s="9" t="n"/>
+      <c r="D102" s="9" t="n"/>
       <c r="E102" s="9" t="inlineStr">
         <is>
           <t>deg</t>
         </is>
       </c>
       <c r="F102" s="8" t="n"/>
-      <c r="G102" s="11">
-        <f>IF(AND(ISNUMBER(G95),ISNUMBER(G101),G95&gt;0),ROUND(DEGREES(ATAN((G101-IF(ISNUMBER(G99),G99,D99))/G95)),1),"")</f>
-        <v/>
-      </c>
+      <c r="G102" s="10" t="n"/>
       <c r="H102" s="9">
-        <f>IF(ISNUMBER(G102),G102-D102,"")</f>
+        <f>IF(NOT(ISNUMBER(D102)),"",IF(ISNUMBER(G102),G102-D102,IF(ISNUMBER(F102),F102-D102,"")))</f>
         <v/>
       </c>
       <c r="I102" s="9" t="n"/>
       <c r="J102" s="11">
-        <f>IF(NOT(ISNUMBER(G102)),"",IF(OR(G102&gt;D102,G102&lt;-15),"OVER LIMIT","ok"))</f>
+        <f>IF(OR(H102="",I102=""),"",IF(ABS(H102)&gt;I102,IF(ISNUMBER(G102),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
       <c r="K102" s="5" t="inlineStr">
         <is>
-          <t>Computed. Limit is cone_tilt (12) up and aim_max (15) down before the light cone clips the visor or the body hits the head. OVER LIMIT means a riser, the tripod or a longer throw. Do not type here.</t>
+          <t>Adds to the tilt. Shim the feet.</t>
         </is>
       </c>
     </row>
@@ -4394,14 +4386,14 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Ground slope at the case position</t>
+          <t>Distance from the case to where visitors first appear</t>
         </is>
       </c>
       <c r="C103" s="9" t="n"/>
       <c r="D103" s="9" t="n"/>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>deg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="F103" s="8" t="n"/>
@@ -4417,7 +4409,7 @@
       </c>
       <c r="K103" s="5" t="inlineStr">
         <is>
-          <t>Adds to the tilt. Shim the feet or use the tripod.</t>
+          <t>HC-SR501 range is about 7 m. Sets the PIR sensitivity and whether the rear wall is the right face for it.</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4421,7 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>Distance from the case to where visitors first appear</t>
+          <t>Distance from the case to the GFCI outlet</t>
         </is>
       </c>
       <c r="C104" s="9" t="n"/>
@@ -4452,160 +4444,82 @@
       </c>
       <c r="K104" s="5" t="inlineStr">
         <is>
-          <t>HC-SR501 range is about 7 m. Sets the PIR sensitivity and whether the rear wall is the right face for it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="9" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="inlineStr">
-        <is>
-          <t>Distance from the case to the GFCI outlet</t>
-        </is>
-      </c>
-      <c r="C105" s="9" t="n"/>
-      <c r="D105" s="9" t="n"/>
-      <c r="E105" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="F105" s="8" t="n"/>
-      <c r="G105" s="10" t="n"/>
-      <c r="H105" s="9">
-        <f>IF(NOT(ISNUMBER(D105)),"",IF(ISNUMBER(G105),G105-D105,IF(ISNUMBER(F105),F105-D105,"")))</f>
-        <v/>
-      </c>
-      <c r="I105" s="9" t="n"/>
-      <c r="J105" s="11">
-        <f>IF(OR(H105="",I105=""),"",IF(ABS(H105)&gt;I105,IF(ISNUMBER(G105),"UPDATE","UPDATE (spec)"),"ok"))</f>
-        <v/>
-      </c>
-      <c r="K105" s="5" t="inlineStr">
-        <is>
           <t>One AC cord, under a cord cover across any path. Sets its length.</t>
         </is>
       </c>
     </row>
+    <row r="105"/>
     <row r="106">
-      <c r="A106" s="9" t="inlineStr">
-        <is>
-          <t>Assembly</t>
-        </is>
-      </c>
-      <c r="B106" s="5" t="inlineStr">
-        <is>
-          <t>Centre of mass behind the footprint centre (+ = rear)</t>
-        </is>
-      </c>
-      <c r="C106" s="9" t="inlineStr">
-        <is>
-          <t>tripod_y</t>
-        </is>
-      </c>
-      <c r="D106" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="E106" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="F106" s="8" t="n"/>
-      <c r="G106" s="10" t="n"/>
-      <c r="H106" s="9">
-        <f>IF(NOT(ISNUMBER(D106)),"",IF(ISNUMBER(G106),G106-D106,IF(ISNUMBER(F106),F106-D106,"")))</f>
-        <v/>
-      </c>
-      <c r="I106" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="J106" s="11">
-        <f>IF(OR(H106="",I106=""),"",IF(ABS(H106)&gt;I106,IF(ISNUMBER(G106),"UPDATE","UPDATE (spec)"),"ok"))</f>
-        <v/>
-      </c>
-      <c r="K106" s="5" t="inlineStr">
-        <is>
-          <t>Loaded case, lid on: balance it on a rod across the feet, mark the line, measure from the footprint centre. Move tripod_y and reprint the base rear tile only if it moves more than the tolerance.</t>
-        </is>
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>Parameters to update</t>
+        </is>
+      </c>
+      <c r="B106" s="6">
+        <f>COUNTIF(J7:J104,"UPDATE*")+COUNTIF(J7:J104,"OVER LIMIT")</f>
+        <v/>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>Rows still blank</t>
+        </is>
+      </c>
+      <c r="D106" s="6">
+        <f>COUNTBLANK(G7:G104)</f>
+        <v/>
       </c>
     </row>
     <row r="107"/>
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>Parameters to update</t>
-        </is>
-      </c>
-      <c r="B108" s="6">
-        <f>COUNTIF(J7:J106,"UPDATE*")+COUNTIF(J7:J106,"OVER LIMIT")</f>
-        <v/>
-      </c>
-      <c r="C108" s="6" t="inlineStr">
-        <is>
-          <t>Rows still blank</t>
-        </is>
-      </c>
-      <c r="D108" s="6">
-        <f>COUNTBLANK(G7:G106)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="109"/>
+          <t>Legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Yellow cell</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Type your measurement here.</t>
+        </is>
+      </c>
+    </row>
     <row r="110">
-      <c r="A110" s="6" t="inlineStr">
-        <is>
-          <t>Legend</t>
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>Green value</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>From the Tkisko TO2 manual (manuals.plus, Oct 2022), its label and product photos. Confirm with calipers.</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>Yellow cell</t>
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>Bold value</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Type your measurement here.</t>
+          <t>Computed by the sheet. Leave it alone.</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="8" t="inlineStr">
-        <is>
-          <t>Green value</t>
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Defaults and tolerances</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
-        <is>
-          <t>From the Tkisko TO2 manual (manuals.plus, Oct 2022), its label and product photos. Confirm with calipers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="6" t="inlineStr">
-        <is>
-          <t>Bold value</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t>Computed by the sheet. Leave it alone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>Defaults and tolerances</t>
-        </is>
-      </c>
-      <c r="B114" s="4" t="inlineStr">
         <is>
           <t>Taken from projector_pi_case.scad (v0.9 draft) and docs/BRINGUP.md. The weight default (720 g) is an assumption from the design log, not a measurement. Site rows and the Assembly row are about where the case will stand, not the hardware: fill them before printing the big tiles.</t>
         </is>
@@ -4622,7 +4536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5212,7 +5126,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>3/8-16 insert fit</t>
+          <t>1/4-20 insert fit</t>
         </is>
       </c>
       <c r="C30" s="8" t="n"/>
@@ -5231,7 +5145,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>1/4-20 insert fit</t>
+          <t>M4 insert fit</t>
         </is>
       </c>
       <c r="C31" s="8" t="n"/>
@@ -5250,7 +5164,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>M4 insert fit</t>
+          <t>M3 insert fit</t>
         </is>
       </c>
       <c r="C32" s="8" t="n"/>
@@ -5269,14 +5183,14 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>M3 insert fit</t>
+          <t>M3 / M2.5 / M2 screws in the pilots</t>
         </is>
       </c>
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="10" t="n"/>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>snug / loose / cracked</t>
+          <t>bite / strip / split</t>
         </is>
       </c>
     </row>
@@ -5288,16 +5202,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>M3 / M2.5 / M2 screws in the pilots</t>
+          <t>M4 bolt in the keyhole: slides and seats?</t>
         </is>
       </c>
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="10" t="n"/>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>bite / strip / split</t>
-        </is>
-      </c>
+      <c r="E34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
@@ -5307,27 +5217,12 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>M4 bolt in the keyhole: slides and seats?</t>
+          <t>Acrylic in the slot: snug, no rattle?</t>
         </is>
       </c>
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="10" t="n"/>
       <c r="E35" s="5" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>Fit coupon</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Acrylic in the slot: snug, no rattle?</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="n"/>
-      <c r="D36" s="10" t="n"/>
-      <c r="E36" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Review fixes: louver slots inside caps, baffle to floor, stale worksheet and docs
air_n floors (9 and 6 slats) with extent asserts, baffle runs to the floor,
in_right dropped, measurements.xlsx repointed to the airflow parameters,
v0.10 labels, HDMI/DC plug and IR holder assembly notes, upgrade note.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/measurements.xlsx
+++ b/docs/measurements.xlsx
@@ -519,6 +519,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
@@ -983,12 +984,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Lowest plug edge above underside</t>
+          <t>DC jack centre: inset from the right edge (rear face, top-right corner)</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>port_band[0]</t>
+          <t>dc_jack[0]</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
@@ -999,14 +1000,16 @@
           <t>mm</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n"/>
+      <c r="F15" s="8" t="n">
+        <v>15</v>
+      </c>
       <c r="G15" s="10" t="n"/>
       <c r="H15" s="9">
         <f>IF(NOT(ISNUMBER(D15)),"",IF(ISNUMBER(G15),G15-D15,IF(ISNUMBER(F15),F15-D15,"")))</f>
         <v/>
       </c>
       <c r="I15" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J15" s="11">
         <f>IF(OR(H15="",I15=""),"",IF(ABS(H15)&gt;I15,IF(ISNUMBER(G15),"UPDATE","UPDATE (spec)"),"ok"))</f>
@@ -1014,7 +1017,7 @@
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>With the HDMI and power plugs fitted.</t>
+          <t>Photo-derived (2026-10-06 owner photos); confirm with calipers. Barrel centre, measured from the projector's right edge.</t>
         </is>
       </c>
     </row>
@@ -1026,36 +1029,42 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Highest plug edge above underside</t>
+          <t>DC jack centre: below the projector's top</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>port_band[1]</t>
+          <t>dc_jack[1]</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F16" s="8" t="n"/>
+      <c r="F16" s="8" t="n">
+        <v>13</v>
+      </c>
       <c r="G16" s="10" t="n"/>
       <c r="H16" s="9">
         <f>IF(NOT(ISNUMBER(D16)),"",IF(ISNUMBER(G16),G16-D16,IF(ISNUMBER(F16),F16-D16,"")))</f>
         <v/>
       </c>
       <c r="I16" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J16" s="11">
         <f>IF(OR(H16="",I16=""),"",IF(ABS(H16)&gt;I16,IF(ISNUMBER(G16),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K16" s="5" t="n"/>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Photo-derived (2026-10-06 owner photos); confirm with calipers. Barrel centre, measured down from the top edge. Sets the DC plug keep-out; the plug must point back and stay above the intake patch.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -1096,7 +1105,7 @@
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>Plugs fitted, cable bent the way it will run. A straight HDMI plug is about 40.</t>
+          <t>Right-angle DC plug standing out of the rear face, cable bent the way it will run. (HDMI is on the right face now, so this is the DC plug only.)</t>
         </is>
       </c>
     </row>
@@ -1108,30 +1117,40 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>HDMI port position along the rear face, X (+ = right)</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
+          <t>HDMI centre behind the front face (right face I/O strip)</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>hdmi_y</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>56</v>
+      </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F18" s="8" t="n"/>
+      <c r="F18" s="8" t="n">
+        <v>56</v>
+      </c>
       <c r="G18" s="10" t="n"/>
       <c r="H18" s="9">
         <f>IF(NOT(ISNUMBER(D18)),"",IF(ISNUMBER(G18),G18-D18,IF(ISNUMBER(F18),F18-D18,"")))</f>
         <v/>
       </c>
-      <c r="I18" s="9" t="n"/>
+      <c r="I18" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="J18" s="11">
         <f>IF(OR(H18="",I18=""),"",IF(ABS(H18)&gt;I18,IF(ISNUMBER(G18),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>Centre of the port. The Pi's cable comes through the divider pass-through (pass_x: -40 to 25 from centre); a port far outside that band means a tight bend behind the projector.</t>
+          <t>Photo-derived (2026-10-06 owner photos); confirm with calipers. The strip spans about 41-118 mm behind the front face; measure the HDMI port centre. Sets the plug keep-out (side_port_*) and where the baffle stands.</t>
         </is>
       </c>
     </row>
@@ -1143,30 +1162,40 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Power jack position along the rear face, X (+ = right)</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
+          <t>Right-face I/O strip height, from the top</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>side_port_h</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>18</v>
+      </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F19" s="8" t="n"/>
+      <c r="F19" s="8" t="n">
+        <v>18</v>
+      </c>
       <c r="G19" s="10" t="n"/>
       <c r="H19" s="9">
         <f>IF(NOT(ISNUMBER(D19)),"",IF(ISNUMBER(G19),G19-D19,IF(ISNUMBER(F19),F19-D19,"")))</f>
         <v/>
       </c>
-      <c r="I19" s="9" t="n"/>
+      <c r="I19" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="J19" s="11">
         <f>IF(OR(H19="",I19=""),"",IF(ABS(H19)&gt;I19,IF(ISNUMBER(G19),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>Centre of the jack.</t>
+          <t>Photo-derived (2026-10-06 owner photos); confirm with calipers. Top strip holding HDMI, USB and AV. Sets baffle_gap (the baffle stops this + 4 mm below the top) and the HDMI cable keep-out.</t>
         </is>
       </c>
     </row>
@@ -1396,17 +1425,25 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>IR receiver window height above underside</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
+          <t>IR receiver window height above underside (front face, above the logo)</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>ir_z</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>50</v>
+      </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F26" s="8" t="n"/>
+      <c r="F26" s="8" t="n">
+        <v>50</v>
+      </c>
       <c r="G26" s="10" t="n"/>
       <c r="H26" s="9">
         <f>IF(NOT(ISNUMBER(D26)),"",IF(ISNUMBER(G26),G26-D26,IF(ISNUMBER(F26),F26-D26,"")))</f>
@@ -1421,7 +1458,7 @@
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>ir_holder sticks on inside the case and aims a 5 mm LED ir_angle (30 deg) at this window. Face in Observations.</t>
+          <t>Photo-derived (2026-10-06 owner photos); confirm with calipers. ir_holder sticks on the projector's front face here, body pointing toward the window; it fires at the receiver from inside the front gap.</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1470,25 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>IR receiver position along its face (+ = right)</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
+          <t>IR receiver position along the front face, X (+ = right of centre)</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>ir_x</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>35</v>
+      </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F27" s="8" t="n"/>
+      <c r="F27" s="8" t="n">
+        <v>35</v>
+      </c>
       <c r="G27" s="10" t="n"/>
       <c r="H27" s="9">
         <f>IF(NOT(ISNUMBER(D27)),"",IF(ISNUMBER(G27),G27-D27,IF(ISNUMBER(F27),F27-D27,"")))</f>
@@ -1456,7 +1501,11 @@
         <f>IF(OR(H27="",I27=""),"",IF(ABS(H27)&gt;I27,IF(ISNUMBER(G27),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K27" s="5" t="n"/>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Photo-derived (2026-10-06 owner photos); confirm with calipers. Measure from the body centre.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -1466,24 +1515,32 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Intake vent extent along its face (from-to, + = right)</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
+          <t>Rear intake patch: size (square)</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>in_size</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>40</v>
+      </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F28" s="8" t="n"/>
+      <c r="F28" s="8" t="n">
+        <v>40</v>
+      </c>
       <c r="G28" s="10" t="n"/>
       <c r="H28" s="9">
         <f>IF(NOT(ISNUMBER(D28)),"",IF(ISNUMBER(G28),G28-D28,IF(ISNUMBER(F28),F28-D28,"")))</f>
         <v/>
       </c>
       <c r="I28" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J28" s="11">
         <f>IF(OR(H28="",I28=""),"",IF(ABS(H28)&gt;I28,IF(ISNUMBER(G28),"UPDATE","UPDATE (spec)"),"ok"))</f>
@@ -1491,7 +1548,7 @@
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>Type as from-to, e.g. -70-(-20). Louver banks (vents) and the floor intake should feed it. Face in Observations.</t>
+          <t>Photo-derived (2026-10-06 owner photos); confirm with calipers. The rear-face grille the inlet bank feeds; the speaker grille beside it is not an air path. Sizes the inlet opening.</t>
         </is>
       </c>
     </row>
@@ -1503,30 +1560,42 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Intake vent height band above underside (low-high)</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
+          <t>Rear intake patch: inset from the projector's top</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>in_top</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>15</v>
+      </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F29" s="8" t="n"/>
+      <c r="F29" s="8" t="n">
+        <v>15</v>
+      </c>
       <c r="G29" s="10" t="n"/>
       <c r="H29" s="9">
         <f>IF(NOT(ISNUMBER(D29)),"",IF(ISNUMBER(G29),G29-D29,IF(ISNUMBER(F29),F29-D29,"")))</f>
         <v/>
       </c>
       <c r="I29" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J29" s="11">
         <f>IF(OR(H29="",I29=""),"",IF(ABS(H29)&gt;I29,IF(ISNUMBER(G29),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K29" s="5" t="n"/>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>Photo-derived (2026-10-06 owner photos); confirm with calipers. Sets the inlet bank's height on the right wall.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -1536,24 +1605,32 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Exhaust vent extent along its face (from-to, + = right)</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
+          <t>Exhaust grille start, behind the front face (right face)</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>exh_y[0]</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F30" s="8" t="n"/>
+      <c r="F30" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="G30" s="10" t="n"/>
       <c r="H30" s="9">
         <f>IF(NOT(ISNUMBER(D30)),"",IF(ISNUMBER(G30),G30-D30,IF(ISNUMBER(F30),F30-D30,"")))</f>
         <v/>
       </c>
       <c r="I30" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J30" s="11">
         <f>IF(OR(H30="",I30=""),"",IF(ABS(H30)&gt;I30,IF(ISNUMBER(G30),"UPDATE","UPDATE (spec)"),"ok"))</f>
@@ -1561,7 +1638,7 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>The projector-zone 40 mm fan on the right wall should sit level with it. Face in Observations.</t>
+          <t>Photo-derived (2026-10-06 owner photos); confirm with calipers. Slots measured 10-42 mm; the owner says the first 40. Sets the exhaust bank's position.</t>
         </is>
       </c>
     </row>
@@ -1573,30 +1650,42 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Exhaust vent height band above underside (low-high)</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
+          <t>Exhaust grille end, behind the front face (right face)</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>exh_y[1]</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>42</v>
+      </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F31" s="8" t="n"/>
+      <c r="F31" s="8" t="n">
+        <v>42</v>
+      </c>
       <c r="G31" s="10" t="n"/>
       <c r="H31" s="9">
         <f>IF(NOT(ISNUMBER(D31)),"",IF(ISNUMBER(G31),G31-D31,IF(ISNUMBER(F31),F31-D31,"")))</f>
         <v/>
       </c>
       <c r="I31" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J31" s="11">
         <f>IF(OR(H31="",I31=""),"",IF(ABS(H31)&gt;I31,IF(ISNUMBER(G31),"UPDATE","UPDATE (spec)"),"ok"))</f>
         <v/>
       </c>
-      <c r="K31" s="5" t="n"/>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>Sets the exhaust opening length (with air_margin each end). The grille spans the full projector height.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
@@ -1683,11 +1772,7 @@
           <t>Weight</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="C34" s="9" t="inlineStr"/>
       <c r="D34" s="9" t="n">
         <v>720</v>
       </c>
@@ -2565,7 +2650,7 @@
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t>Projector label reads DC 21 V (confirm with a meter). Amp4 takes 12-24 V; fans must be 24 V parts.</t>
+          <t>Projector label reads DC 21 V (confirm with a meter). The second wall-wart's rail is 12-24 V (the DigiAMP+'s range).</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2689,7 @@
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
-          <t>Label: 48 W, 21 V 2.28 A. Model MX48CC-210228US. Covers the projector alone; a second 24 V wall-wart on the upper receptacle feeds the Pi, Amp4 and fans. Sizes the 21 V fuse.</t>
+          <t>Label: 48 W, 21 V 2.28 A. Model MX48CC-210228US. Covers the projector alone; a second 12-24 V wall-wart on the upper receptacle feeds the Pi and the DigiAMP+. Sizes the 21 V fuse.</t>
         </is>
       </c>
     </row>
@@ -2793,7 +2878,7 @@
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t>One on the AC live, one per DC rail (21 V projector, 24 V Pi/Amp4/fans). Type L x D. The AC one sits behind the receptacle plate, the DC ones on the low-voltage side.</t>
+          <t>One on the AC live, one per DC rail (21 V projector, 12-24 V Pi/DigiAMP+). Type L x D. The AC one sits behind the receptacle plate, the DC ones on the low-voltage side.</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2948,7 @@
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t>Feeds the projector plug and the Amp4.</t>
+          <t>Feeds the projector plug and the DigiAMP+.</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2960,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Pi 3/4: board bottom to top of Amp4</t>
+          <t>Pi 3/4: board bottom to top of DigiAMP+</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
@@ -2918,7 +3003,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Pi 5 + Active Cooler: board bottom to top of Amp4</t>
+          <t>Pi 5 + Active Cooler: board bottom to top of DigiAMP+</t>
         </is>
       </c>
       <c r="C66" s="9" t="inlineStr">
@@ -2957,7 +3042,7 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Zero 2 W: board bottom to top of Amp4</t>
+          <t>Zero 2 W: board bottom to top of DigiAMP+</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
@@ -3155,29 +3240,37 @@
     <row r="72">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>Pi stack</t>
+          <t>Airflow</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>DS18B20 probe diameter</t>
-        </is>
-      </c>
-      <c r="C72" s="9" t="n"/>
-      <c r="D72" s="9" t="n"/>
+          <t>HDMI plug standing out of the right face</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>side_port_depth</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="n">
+        <v>15</v>
+      </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F72" s="8" t="n"/>
+      <c r="F72" s="8" t="n">
+        <v>15</v>
+      </c>
       <c r="G72" s="10" t="n"/>
       <c r="H72" s="9">
         <f>IF(NOT(ISNUMBER(D72)),"",IF(ISNUMBER(G72),G72-D72,IF(ISNUMBER(F72),F72-D72,"")))</f>
         <v/>
       </c>
       <c r="I72" s="9" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="J72" s="11">
         <f>IF(OR(H72="",I72=""),"",IF(ABS(H72)&gt;I72,IF(ISNUMBER(G72),"UPDATE","UPDATE (spec)"),"ok"))</f>
@@ -3185,42 +3278,44 @@
       </c>
       <c r="K72" s="5" t="inlineStr">
         <is>
-          <t>Two sensors: projector zone and Pi zone. Sets the clip or hole that holds each probe.</t>
+          <t>Right-angle (side-exit) plug fitted, cable leaving rearward along the face. The keep-out is 16 mm along Y.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>Fans</t>
+          <t>Airflow</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>Fan frame size</t>
+          <t>HDMI cable run behind the plug, standing out of the right face</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>fan</t>
+          <t>side_cable_d</t>
         </is>
       </c>
       <c r="D73" s="9" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F73" s="8" t="n"/>
+      <c r="F73" s="8" t="n">
+        <v>8</v>
+      </c>
       <c r="G73" s="10" t="n"/>
       <c r="H73" s="9">
         <f>IF(NOT(ISNUMBER(D73)),"",IF(ISNUMBER(G73),G73-D73,IF(ISNUMBER(F73),F73-D73,"")))</f>
         <v/>
       </c>
       <c r="I73" s="9" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J73" s="11">
         <f>IF(OR(H73="",I73=""),"",IF(ABS(H73)&gt;I73,IF(ISNUMBER(G73),"UPDATE","UPDATE (spec)"),"ok"))</f>
@@ -3228,31 +3323,37 @@
       </c>
       <c r="K73" s="5" t="inlineStr">
         <is>
-          <t>40 mm fans have 32 mm hole spacing.</t>
+          <t>Cable diameter plus its bend, running rearward over the baffle to the divider pass-through.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>Fans</t>
+          <t>Airflow</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Fan body thickness</t>
-        </is>
-      </c>
-      <c r="C74" s="9" t="n"/>
+          <t>Exhaust/inlet opening margin along Y</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>air_margin</t>
+        </is>
+      </c>
       <c r="D74" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F74" s="8" t="n"/>
+      <c r="F74" s="8" t="n">
+        <v>8</v>
+      </c>
       <c r="G74" s="10" t="n"/>
       <c r="H74" s="9">
         <f>IF(NOT(ISNUMBER(D74)),"",IF(ISNUMBER(G74),G74-D74,IF(ISNUMBER(F74),F74-D74,"")))</f>
@@ -3267,36 +3368,44 @@
       </c>
       <c r="K74" s="5" t="inlineStr">
         <is>
-          <t>fan_body() is 10 thick; with screen and bosses it stands 14 proud of the right wall inside side_air (25). A 20 mm fan clashes with the pan sweep.</t>
+          <t>Partial margin for the pan sweep: at the extremes some exhaust leaves into the side gap, which is the plenum. Not a measurement.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>Fans</t>
+          <t>Airflow</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Fan cable length</t>
-        </is>
-      </c>
-      <c r="C75" s="9" t="n"/>
-      <c r="D75" s="9" t="n"/>
+          <t>Exhaust/inlet opening margin along Z</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>air_margin_z</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="n">
+        <v>4</v>
+      </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="F75" s="8" t="n"/>
+      <c r="F75" s="8" t="n">
+        <v>4</v>
+      </c>
       <c r="G75" s="10" t="n"/>
       <c r="H75" s="9">
         <f>IF(NOT(ISNUMBER(D75)),"",IF(ISNUMBER(G75),G75-D75,IF(ISNUMBER(F75),F75-D75,"")))</f>
         <v/>
       </c>
       <c r="I75" s="9" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="J75" s="11">
         <f>IF(OR(H75="",I75=""),"",IF(ABS(H75)&gt;I75,IF(ISNUMBER(G75),"UPDATE","UPDATE (spec)"),"ok"))</f>
@@ -3304,38 +3413,44 @@
       </c>
       <c r="K75" s="5" t="inlineStr">
         <is>
-          <t>Fan to the Pi header (PWM, tach) and to the splice for 21 V.</t>
+          <t>Partial margin for the tilt sweep, same caveat. Not a measurement.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>Fans</t>
+          <t>Airflow</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Rated voltage</t>
-        </is>
-      </c>
-      <c r="C76" s="9" t="n"/>
+          <t>Side gap each side of the projector</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>side_air</t>
+        </is>
+      </c>
       <c r="D76" s="9" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="F76" s="8" t="n"/>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F76" s="8" t="n">
+        <v>25</v>
+      </c>
       <c r="G76" s="10" t="n"/>
       <c r="H76" s="9">
         <f>IF(NOT(ISNUMBER(D76)),"",IF(ISNUMBER(G76),G76-D76,IF(ISNUMBER(F76),F76-D76,"")))</f>
         <v/>
       </c>
       <c r="I76" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J76" s="11">
         <f>IF(OR(H76="",I76=""),"",IF(ABS(H76)&gt;I76,IF(ISNUMBER(G76),"UPDATE","UPDATE (spec)"),"ok"))</f>
@@ -3343,7 +3458,7 @@
       </c>
       <c r="K76" s="5" t="inlineStr">
         <is>
-          <t>Must be 24 V parts on the 21 V rail; a 12 V fan burns. Check the datasheet's minimum voltage too.</t>
+          <t>Clears the pan sweep of the right face, the HDMI plug and the baffle. Could shrink to about 19 mm (a separate change that moves the base size).</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4864,7 @@
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Taken from projector_pi_case.scad (v0.9 draft) and docs/BRINGUP.md. The weight default (720 g) is an assumption from the design log, not a measurement. Site rows and the Assembly row are about where the case will stand, not the hardware: fill them before printing the big tiles.</t>
+          <t>Taken from projector_pi_case.scad (v0.10 draft) and docs/BRINGUP.md. The weight default (720 g) is an assumption from the design log, not a measurement. Site rows and the Assembly row are about where the case will stand, not the hardware: fill them before printing the big tiles.</t>
         </is>
       </c>
     </row>
@@ -4788,6 +4903,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -4878,13 +4994,13 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Ports: HDMI, USB, AV, 3.5 mm audio. Location not stated.</t>
+          <t>Ports: HDMI, USB, AV, 3.5 mm audio. Photos (2026-10-06): DC jack at the rear top-right corner; HDMI/USB/AV in a strip on the right face.</t>
         </is>
       </c>
       <c r="D7" s="10" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Design assumes the rear face (port_band).</t>
+          <t>The model assumes this (dc_jack, hdmi_y, side_port_*, port_depth). Confirm with calipers.</t>
         </is>
       </c>
     </row>
@@ -4907,7 +5023,7 @@
       <c r="D8" s="10" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Straight HDMI needs about 40 mm of rear_gap.</t>
+          <t>HDMI must be a right-angle, side-exit plug with the cable leaving rearward along the right face: a straight plug does not fit the side gap. The DC plug points back, above the intake patch.</t>
         </is>
       </c>
     </row>
@@ -4943,13 +5059,13 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Sealed optical engine; fan cooling. Locations not stated.</t>
+          <t>Sealed optical engine; fan cooling. Photos: exhaust grille on the right face (first 40 mm behind the front), intake grille on the rear face; the rear face's second grille is a speaker.</t>
         </is>
       </c>
       <c r="D10" s="10" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Louvers and the 40 mm fan should line up with them.</t>
+          <t>The exhaust and inlet louver banks line up with them (exh_y, in_size, in_top).</t>
         </is>
       </c>
     </row>
@@ -4989,13 +5105,13 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Remote included.</t>
+          <t>Remote included. Photos: the receiver window is on the front face, above the logo.</t>
         </is>
       </c>
       <c r="D12" s="10" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>ir_holder sticks on inside the case facing it; a front-face receiver sees nothing from inside.</t>
+          <t>ir_holder sticks on the projector's front face (ir_x, ir_z) with its body pointing toward the window, so the LED fires at the receiver from inside the front gap.</t>
         </is>
       </c>
     </row>
@@ -5012,13 +5128,13 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Sealed optical engine; fan cooling.</t>
+          <t>Sealed optical engine; fan cooling. Photos: exhaust right face, intake rear face.</t>
         </is>
       </c>
       <c r="D13" s="10" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Intake should see the floor slots and louvers; exhaust should see the right-wall fan.</t>
+          <t>The case has no fans: the projector's own fan moves the air. The inlet bank sees the rear intake, the exhaust bank the right-face exhaust.</t>
         </is>
       </c>
     </row>
@@ -5236,13 +5352,13 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Can it run projector + Pi + Amp4 together at full volume?</t>
+          <t>Can it run projector + Pi + DigiAMP+ together at full volume?</t>
         </is>
       </c>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>No: 48 W covers the projector alone. A second 24 V wall-wart (2.5-3 A) on the upper receptacle feeds the Pi, Amp4 and fans.</t>
+          <t>No: 48 W covers the projector alone. A second 12-24 V wall-wart (2.5-3 A) on the upper receptacle feeds the Pi and the DigiAMP+.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -5297,14 +5413,14 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>GPIOs the Amp4 leaves free</t>
+          <t>GPIOs the DigiAMP+ leaves free</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="10" t="n"/>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Needed for PIR, DS18B20s, fan PWM and tach, relay.</t>
+          <t>Needed for the PIR, the relay and the IR LED.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BOM, bring-up rows 4/4a/4b/17a, assembly, printing and worksheet for the brick
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/measurements.xlsx
+++ b/docs/measurements.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Measurements" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Observations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -2481,21 +2481,21 @@
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>Wall-wart</t>
+          <t>Power brick</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Stock wall-wart length (X on the shelf)</t>
+          <t>Brick length (X on the shelf)</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>wart_l</t>
+          <t>brick[0]</t>
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>86</v>
+        <v>150</v>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
@@ -2503,9 +2503,7 @@
         </is>
       </c>
       <c r="F53" s="8" t="n"/>
-      <c r="G53" s="10" t="n">
-        <v>85.59999999999999</v>
-      </c>
+      <c r="G53" s="10" t="n"/>
       <c r="H53" s="9">
         <f>IF(NOT(ISNUMBER(D53)),"",IF(ISNUMBER(G53),G53-D53,IF(ISNUMBER(F53),F53-D53,"")))</f>
         <v/>
@@ -2519,28 +2517,28 @@
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t>Hangs on the shelf receptacle plate standing on its long edge, cord end toward the barrier. 85.6 by caliper (photo, 2026-10-05).</t>
+          <t>PROVISIONAL (typical 120 W desktop brick). Measure the Parts Express brick with calipers on arrival.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>Wall-wart</t>
+          <t>Power brick</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Width = standing height (Z)</t>
+          <t>Brick width (Y on the shelf)</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>wart_w</t>
+          <t>brick[1]</t>
         </is>
       </c>
       <c r="D54" s="9" t="n">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
@@ -2548,9 +2546,7 @@
         </is>
       </c>
       <c r="F54" s="8" t="n"/>
-      <c r="G54" s="10" t="n">
-        <v>47</v>
-      </c>
+      <c r="G54" s="10" t="n"/>
       <c r="H54" s="9">
         <f>IF(NOT(ISNUMBER(D54)),"",IF(ISNUMBER(G54),G54-D54,IF(ISNUMBER(F54),F54-D54,"")))</f>
         <v/>
@@ -2564,28 +2560,28 @@
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>Scaled off the 2026-10-05 photo against the 85.6 caliper reading; confirm with calipers. The two-wart stack has about 3 mm under the lid roof, asserted.</t>
+          <t>PROVISIONAL (typical 120 W desktop brick). Measure the Parts Express brick with calipers on arrival.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>Wall-wart</t>
+          <t>Power brick</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Thickness, prong face to back (Y)</t>
+          <t>Brick height (Z)</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>wart_t</t>
+          <t>brick[2]</t>
         </is>
       </c>
       <c r="D55" s="9" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
@@ -2607,7 +2603,7 @@
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t>Not measured yet. Body only, prongs excluded. Sets how far the warts hang off the plate toward the divider.</t>
+          <t>PROVISIONAL (typical 120 W desktop brick). Measure the Parts Express brick with calipers on arrival.</t>
         </is>
       </c>
     </row>
@@ -2650,7 +2646,7 @@
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t>Projector label reads DC 21 V (confirm with a meter). The second wall-wart's rail is 12-24 V (the DigiAMP+'s range).</t>
+          <t>Brick: 24 V (Parts Express). Projector label 21 V: BRINGUP row 4a</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2685,7 @@
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
-          <t>Label: 48 W, 21 V 2.28 A. Model MX48CC-210228US. Covers the projector alone; a second 12-24 V wall-wart on the upper receptacle feeds the Pi and the DigiAMP+. Sizes the 21 V fuse.</t>
+          <t>Brick: 5 A (120 W). Read the label</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2722,7 @@
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t>Label: AC 100-240 V 50/60 Hz 1.0 A max. Add the second wall-wart's input current; sizes the AC fuse (3 A T).</t>
+          <t>Read the brick's label (no AC fuse is fitted)</t>
         </is>
       </c>
     </row>
@@ -3718,16 +3714,16 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>Cord grip panel hole</t>
+          <t>Cord opening in the rear wall (X)</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>gland_d</t>
+          <t>cord_open[0]</t>
         </is>
       </c>
       <c r="D83" s="9" t="n">
-        <v>15.5</v>
+        <v>40</v>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
@@ -3749,7 +3745,7 @@
       </c>
       <c r="K83" s="5" t="inlineStr">
         <is>
-          <t>PG9 is 15.2 nominal; take it from the grip's datasheet.</t>
+          <t>Must pass the cord's molded connector with room (a C13 body is about 28 x 21 mm). Measure yours.</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4787,6 @@
         </is>
       </c>
     </row>
-    <row r="111"/>
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
@@ -4812,7 +4807,6 @@
         <v/>
       </c>
     </row>
-    <row r="113"/>
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
@@ -4903,7 +4897,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -5358,12 +5351,12 @@
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>No: 48 W covers the projector alone. A second 12-24 V wall-wart (2.5-3 A) on the upper receptacle feeds the Pi and the DigiAMP+.</t>
+          <t>Replaced by the Parts Express 24 V 5 A (120 W) brick, which covers all three. Projector tolerance of 24 V: BRINGUP row 4a.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Bench test; watch for undervoltage.</t>
+          <t>BRINGUP rows 4a and 4b.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Worksheet and docs: retire stale wall-wart/fuse/gland rows, fix BOM and print totals
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/measurements.xlsx
+++ b/docs/measurements.xlsx
@@ -519,7 +519,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
@@ -2094,7 +2093,7 @@
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>Manual: 50 W. Sizes the brick and the DC fuse.</t>
+          <t>Manual: 50 W. Compare with the brick's rating (120 W) and the Y-splitter's lead rating.</t>
         </is>
       </c>
     </row>
@@ -2627,12 +2626,8 @@
           <t>V</t>
         </is>
       </c>
-      <c r="F56" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="G56" s="10" t="n">
-        <v>21</v>
-      </c>
+      <c r="F56" s="8" t="n"/>
+      <c r="G56" s="10" t="n"/>
       <c r="H56" s="9">
         <f>IF(NOT(ISNUMBER(D56)),"",IF(ISNUMBER(G56),G56-D56,IF(ISNUMBER(F56),F56-D56,"")))</f>
         <v/>
@@ -2668,12 +2663,8 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F57" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="G57" s="10" t="n">
-        <v>2.28</v>
-      </c>
+      <c r="F57" s="8" t="n"/>
+      <c r="G57" s="10" t="n"/>
       <c r="H57" s="9">
         <f>IF(NOT(ISNUMBER(D57)),"",IF(ISNUMBER(G57),G57-D57,IF(ISNUMBER(F57),F57-D57,"")))</f>
         <v/>
@@ -2708,9 +2699,7 @@
         </is>
       </c>
       <c r="F58" s="8" t="n"/>
-      <c r="G58" s="10" t="n">
-        <v>1</v>
-      </c>
+      <c r="G58" s="10" t="n"/>
       <c r="H58" s="9">
         <f>IF(NOT(ISNUMBER(D58)),"",IF(ISNUMBER(G58),G58-D58,IF(ISNUMBER(F58),F58-D58,"")))</f>
         <v/>
@@ -2739,7 +2728,7 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>(gland_d)</t>
+          <t>cord_d</t>
         </is>
       </c>
       <c r="D59" s="9" t="n"/>
@@ -2749,11 +2738,7 @@
         </is>
       </c>
       <c r="F59" s="8" t="n"/>
-      <c r="G59" s="10" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
+      <c r="G59" s="10" t="n"/>
       <c r="H59" s="9">
         <f>IF(NOT(ISNUMBER(D59)),"",IF(ISNUMBER(G59),G59-D59,IF(ISNUMBER(F59),F59-D59,"")))</f>
         <v/>
@@ -2765,7 +2750,7 @@
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t>Wall-wart with fixed prongs: no AC cord. The outdoor cord (SJTW 18 AWG, 3-wire) goes through the PG9 to the receptacles.</t>
+          <t>Outer diameter of the brick's standard molded AC cord, where it passes the rear-wall opening and the cord clamp. Sets `cord_d` (PROVISIONAL 9). The connector's face size sets `cord_open`.</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2787,7 @@
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t>Has to reach from the shelf, over the divider, to the projector's rear jack at 15 deg up-tilt, with the relay and fuse holder spliced in. Spare goes in a loop on the low-voltage side, not coiled by the brick.</t>
+          <t>Brick's DC cord to the Y-splitter, then the splitter's legs to the projector's rear jack (at 15 deg up-tilt) and to the DigiAMP+. Spare goes in a loop on the low-voltage side, not coiled by the brick. A relay, if built, is spliced in leg 1.</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2799,7 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>AC cord length, brick to gland</t>
+          <t>AC cord length, brick to rear-wall opening</t>
         </is>
       </c>
       <c r="C61" s="9" t="n"/>
@@ -2839,7 +2824,7 @@
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
-          <t>The gland is at cord_x (-94), cord_dz (20) above the shelf, in the rear-left corner beside the receptacle plate. Needs a drip loop inside the case.</t>
+          <t>From the brick's inlet to the opening in the rear wall (`cord_open`) and its clamp. Needs slack inside for the connector and a drip loop outside below the clamp.</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2836,7 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Inline fuse holder length and diameter (x2)</t>
+          <t>RETIRED: no fuses fitted</t>
         </is>
       </c>
       <c r="C62" s="9" t="n"/>
@@ -2874,7 +2859,7 @@
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t>One on the AC live, one per DC rail (21 V projector, 12-24 V Pi/DigiAMP+). Type L x D. The AC one sits behind the receptacle plate, the DC ones on the low-voltage side.</t>
+          <t>No fuses in the single-brick design (the brick is current-limited and short-circuit protected). Row kept so formulas stay aligned; leave blank.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2929,7 @@
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t>Feeds the projector plug and the DigiAMP+.</t>
+          <t>Y-splitter body (5.5 x 2.5 mm, 1 female to 2 male) and any relay splice. Sits on the low-voltage side; feeds the projector adapter and the DigiAMP+.</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5317,7 @@
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>None: wall-wart with fixed NEMA 1-15 prongs (2-pin, non-polarized, Class II). No IEC inlet.</t>
+          <t>Unknown until the Parts Express brick arrives: read its label (BRINGUP row 4) and buy a cord with the matching molded connector.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr"/>

</xml_diff>